<commit_message>
Actualizar archivos Excel de datos fuente
🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
+++ b/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjmax\Downloads\1\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4804A0D-D9CD-4B91-892C-6BDE1C542B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A404D43-5CE9-4FF6-BA4C-5FCA920C09F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26325" yWindow="945" windowWidth="24750" windowHeight="14190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Certificaciones" sheetId="1" r:id="rId1"/>
@@ -491,7 +491,8 @@
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="6" width="11.85546875" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" customWidth="1"/>
     <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Filtrado exhaustivo de facturas: eliminar 2025 de todos los archivos
- Arreglado regenerar_dashboard.py: GG/VEH detail usaba 'fecha de imputacion' (eliminada)
- Añadido filtro año en crear_excel_completo.py para que Excel solo muestre 2026
- Ambos dashboards V1 y V2 ahora muestran 0 facturas de 2025
- Excel actualizado con solo 492 facturas (antes 1071)

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
+++ b/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjmax\Downloads\1\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1EEC8E-D1C6-494F-994F-109B9EDB0FA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A95B8F4-8CAD-4165-BD1D-393155088BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21195" yWindow="915" windowWidth="17550" windowHeight="14190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Certificaciones" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -491,7 +491,7 @@
   <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="1" max="1" width="42.28515625" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" customWidth="1"/>

</xml_diff>

<commit_message>
Cuadra el Excel con el dashboard al anadir obras nuevas
La columna 'Mano de Obra' del Resumen cruzaba los nombres de obra de forma
literal, asi que 25.891 EUR de horas (2100, 2600, 24008 y 26021) se quedaban
fuera de ningun proyecto y el margen del Excel salia 25.891 EUR mas alto que
el del dashboard. Ahora los nombres se llevan al canonico de cada obra por
codigo, igual que ya se hacia con las facturas.

Ademas, la mano de obra del dashboard se empareja ahora por codigo de obra:
sin eso, certificar una obra nueva dejaba sus horas en una ficha aparte sin
certificacion y sus facturas descolgadas. El Excel tolerate que la columna de
total de certificaciones venga sin calcular, y se ignoran los ficheros de
bloqueo ~$ de Excel al publicar.

Cifras verificadas contra el dashboard: certificaciones, gastos directos, mano
de obra y margen coinciden al centimo (el prorrateo difiere en 0,02 por
redondeo).

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
+++ b/dashboard/CERTIFICACIONES POR MESES 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjmax\Downloads\1\dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144366EA-37BF-4FD6-B45A-215991A577FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D962B6-FC87-4148-97A4-F1CFE314CD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25920" yWindow="60" windowWidth="25335" windowHeight="14190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2130" yWindow="630" windowWidth="25335" windowHeight="14190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Certificaciones" sheetId="1" r:id="rId1"/>
@@ -497,7 +497,7 @@
   <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" customWidth="1"/>
+    <col min="1" max="1" width="51.140625" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" customWidth="1"/>

</xml_diff>